<commit_message>
- Removed the minus for expired quantity in supplies list - Added qty expired in the Device and Sites Overview
</commit_message>
<xml_diff>
--- a/api/templates/devices_and_sites_overview/en.xlsx
+++ b/api/templates/devices_and_sites_overview/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\devices_and_sites_overview\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBA5657-AA82-43CA-BE21-7D01413481C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71711033-3729-4CB7-A5A6-C469B5B85F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>&lt;Table&gt;</t>
   </si>
@@ -99,6 +99,12 @@
   </si>
   <si>
     <t>Notes: this report only includes the consumables that were sometime tracked on the sites</t>
+  </si>
+  <si>
+    <t>Quantity On Hand but Expired</t>
+  </si>
+  <si>
+    <t>&lt;quantityExpired&gt;</t>
   </si>
 </sst>
 </file>
@@ -743,9 +749,12 @@
         <v>9</v>
       </c>
       <c r="F8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="H8" s="8" t="s">
         <v>16</v>
       </c>
     </row>
@@ -766,9 +775,12 @@
         <v>12</v>
       </c>
       <c r="F9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="7" t="s">
         <v>17</v>
       </c>
       <c r="O9" s="1"/>

</xml_diff>